<commit_message>
Checkpoint: snapshot before URL flattening migration
Pre-migration state of the prototype with all Phase A+B work complete.
50+ routes, 14 primitives, 69 composites, 8 layouts, 13 data files.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOCS/Incorporate123_Project_Task_List.xlsx
+++ b/DOCS/Incorporate123_Project_Task_List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexo\Downloads\Inc123\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexo\Projects\inc123\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9004BF-1900-4F53-AAED-B09321D2CAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE8FC8E-4228-4FFE-81D8-8BF19405EBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -228,12 +228,6 @@
     <t>#14</t>
   </si>
   <si>
-    <t>Competitive analysis (5 competitors)</t>
-  </si>
-  <si>
-    <t>Deep-dive analysis of ZenBusiness, LegalZoom, Bizee, Northwest RA, and 1 other. Analyze site structure, SEO positioning, package presentation, UX patterns.</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
@@ -1333,6 +1327,12 @@
   </si>
   <si>
     <t>Upon successful launch</t>
+  </si>
+  <si>
+    <t>Competitive analysis</t>
+  </si>
+  <si>
+    <t>Deep-dive analysis. Analyze site structure, SEO positioning, package presentation, UX patterns.</t>
   </si>
 </sst>
 </file>
@@ -1493,6 +1493,25 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1513,25 +1532,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1881,46 +1881,46 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-    </row>
-    <row r="3" spans="1:10" s="28" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="26">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+    </row>
+    <row r="3" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="10">
         <v>1</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="G3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="H3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
     </row>
     <row r="4" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
@@ -2092,33 +2092,33 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" s="28" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="26">
+    <row r="10" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="10">
         <v>8</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="27" t="s">
+      <c r="H10" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
@@ -2148,243 +2148,243 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6">
+    <row r="12" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="10">
         <v>10</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-    </row>
-    <row r="13" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2">
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+    </row>
+    <row r="13" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="10">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-    </row>
-    <row r="15" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="6">
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
+    </row>
+    <row r="15" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="10">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-    </row>
-    <row r="16" spans="1:10" s="28" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="26">
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+    </row>
+    <row r="16" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="10">
         <v>13</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="H16" s="27" t="s">
+      <c r="H16" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I16" s="26"/>
-      <c r="J16" s="26"/>
-    </row>
-    <row r="17" spans="1:10" s="28" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="26">
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+    </row>
+    <row r="17" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="10">
         <v>14</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F17" s="26" t="s">
+      <c r="F17" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="H17" s="27" t="s">
+      <c r="H17" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I17" s="26"/>
-      <c r="J17" s="26"/>
-    </row>
-    <row r="18" spans="1:10" s="28" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="26">
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+    </row>
+    <row r="18" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="10">
         <v>15</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="F18" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-    </row>
-    <row r="19" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="6">
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+    </row>
+    <row r="19" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="10">
         <v>16</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="F19" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+    </row>
+    <row r="20" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="10">
+        <v>17</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="D20" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="E20" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G19" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-    </row>
-    <row r="20" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="2">
-        <v>17</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="G20" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
     </row>
     <row r="21" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6">
@@ -2394,16 +2394,16 @@
         <v>52</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>59</v>
@@ -2414,61 +2414,61 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
     </row>
-    <row r="22" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="2">
+    <row r="22" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="10">
         <v>19</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G22" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="H22" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+    </row>
+    <row r="23" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="10">
+        <v>20</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G22" s="3" t="s">
+      <c r="D23" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="H22" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-    </row>
-    <row r="23" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="6">
-        <v>20</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="E23" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G23" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D23" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
     </row>
     <row r="24" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
@@ -2478,10 +2478,10 @@
         <v>52</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>14</v>
@@ -2490,7 +2490,7 @@
         <v>44</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>32</v>
@@ -2498,33 +2498,33 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="6">
+    <row r="25" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="10">
         <v>22</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G25" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
@@ -2534,10 +2534,10 @@
         <v>52</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>44</v>
@@ -2546,10 +2546,10 @@
         <v>44</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
@@ -2562,10 +2562,10 @@
         <v>52</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>14</v>
@@ -2574,107 +2574,107 @@
         <v>44</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>32</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+    </row>
+    <row r="29" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="10">
+        <v>25</v>
+      </c>
+      <c r="B29" s="11" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="22" t="s">
+      <c r="C29" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-    </row>
-    <row r="29" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="2">
-        <v>25</v>
-      </c>
-      <c r="B29" s="3" t="s">
+      <c r="D29" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="E29" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="G29" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="H29" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+    </row>
+    <row r="30" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="10">
+        <v>26</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E30" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="H29" s="3" t="s">
+      <c r="F30" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-    </row>
-    <row r="30" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6">
-        <v>26</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
     </row>
     <row r="31" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>27</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>58</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>60</v>
@@ -2687,22 +2687,22 @@
         <v>28</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>58</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>60</v>
@@ -2715,22 +2715,22 @@
         <v>29</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="F33" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="G33" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>60</v>
@@ -2743,22 +2743,22 @@
         <v>30</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H34" s="7" t="s">
         <v>60</v>
@@ -2771,22 +2771,22 @@
         <v>31</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>63</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>60</v>
@@ -2799,22 +2799,22 @@
         <v>32</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>63</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H36" s="7" t="s">
         <v>60</v>
@@ -2827,13 +2827,13 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>58</v>
@@ -2842,7 +2842,7 @@
         <v>63</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>60</v>
@@ -2855,22 +2855,22 @@
         <v>34</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>60</v>
@@ -2883,13 +2883,13 @@
         <v>35</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>14</v>
@@ -2898,7 +2898,7 @@
         <v>58</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>32</v>
@@ -2911,22 +2911,22 @@
         <v>36</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>32</v>
@@ -2939,13 +2939,13 @@
         <v>37</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>14</v>
@@ -2954,7 +2954,7 @@
         <v>63</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>32</v>
@@ -2967,13 +2967,13 @@
         <v>38</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>14</v>
@@ -2982,7 +2982,7 @@
         <v>63</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>32</v>
@@ -2995,22 +2995,22 @@
         <v>39</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>44</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>60</v>
@@ -3019,43 +3019,43 @@
       <c r="J43" s="2"/>
     </row>
     <row r="44" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="11"/>
-      <c r="J44" s="11"/>
+      <c r="A44" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="20"/>
     </row>
     <row r="45" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6">
         <v>40</v>
       </c>
       <c r="B45" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D45" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="C45" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>150</v>
-      </c>
       <c r="E45" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>58</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I45" s="6"/>
       <c r="J45" s="6"/>
@@ -3065,25 +3065,25 @@
         <v>41</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C46" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G46" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D46" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>155</v>
-      </c>
       <c r="H46" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
@@ -3093,13 +3093,13 @@
         <v>42</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>14</v>
@@ -3108,7 +3108,7 @@
         <v>63</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H47" s="7" t="s">
         <v>32</v>
@@ -3121,13 +3121,13 @@
         <v>43</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>14</v>
@@ -3136,14 +3136,14 @@
         <v>63</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H48" s="5" t="s">
         <v>32</v>
       </c>
       <c r="I48" s="4"/>
       <c r="J48" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
@@ -3151,25 +3151,25 @@
         <v>44</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C49" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="E49" s="6" t="s">
         <v>163</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>165</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>63</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I49" s="6"/>
       <c r="J49" s="6"/>
@@ -3179,25 +3179,25 @@
         <v>45</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>63</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
@@ -3207,25 +3207,25 @@
         <v>46</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C51" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F51" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="D51" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>171</v>
-      </c>
       <c r="G51" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I51" s="6"/>
       <c r="J51" s="6"/>
@@ -3235,25 +3235,25 @@
         <v>47</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
@@ -3263,25 +3263,25 @@
         <v>48</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I53" s="6"/>
       <c r="J53" s="6"/>
@@ -3291,25 +3291,25 @@
         <v>49</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C54" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G54" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D54" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="H54" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
@@ -3319,25 +3319,25 @@
         <v>50</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I55" s="6"/>
       <c r="J55" s="6"/>
@@ -3347,25 +3347,25 @@
         <v>51</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
@@ -3375,25 +3375,25 @@
         <v>52</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I57" s="6"/>
       <c r="J57" s="6"/>
@@ -3403,25 +3403,25 @@
         <v>53</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
@@ -3431,22 +3431,22 @@
         <v>54</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H59" s="7" t="s">
         <v>32</v>
@@ -3459,29 +3459,29 @@
         <v>55</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H60" s="5" t="s">
         <v>32</v>
       </c>
       <c r="I60" s="4"/>
       <c r="J60" s="4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
@@ -3489,22 +3489,22 @@
         <v>56</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H61" s="7" t="s">
         <v>32</v>
@@ -3517,69 +3517,69 @@
         <v>57</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H62" s="5" t="s">
         <v>32</v>
       </c>
       <c r="I62" s="4"/>
       <c r="J62" s="4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="B63" s="25"/>
-      <c r="C63" s="25"/>
-      <c r="D63" s="25"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="25"/>
-      <c r="G63" s="25"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="25"/>
-      <c r="J63" s="25"/>
+      <c r="A63" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+      <c r="F63" s="18"/>
+      <c r="G63" s="18"/>
+      <c r="H63" s="18"/>
+      <c r="I63" s="18"/>
+      <c r="J63" s="18"/>
     </row>
     <row r="64" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6">
         <v>58</v>
       </c>
       <c r="B64" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D64" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="C64" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="D64" s="7" t="s">
-        <v>208</v>
-      </c>
       <c r="E64" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>58</v>
       </c>
       <c r="G64" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H64" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="6"/>
@@ -3589,25 +3589,25 @@
         <v>59</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>58</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
@@ -3617,25 +3617,25 @@
         <v>60</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H66" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I66" s="6"/>
       <c r="J66" s="6"/>
@@ -3645,25 +3645,25 @@
         <v>61</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
@@ -3673,25 +3673,25 @@
         <v>62</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>63</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H68" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="6"/>
@@ -3701,25 +3701,25 @@
         <v>63</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>63</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
@@ -3729,25 +3729,25 @@
         <v>64</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C70" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="E70" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="D70" s="7" t="s">
+      <c r="F70" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="E70" s="6" t="s">
+      <c r="G70" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="F70" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="G70" s="7" t="s">
-        <v>225</v>
-      </c>
       <c r="H70" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="6"/>
@@ -3757,25 +3757,25 @@
         <v>65</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G71" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D71" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>228</v>
-      </c>
       <c r="H71" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
@@ -3785,25 +3785,25 @@
         <v>66</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C72" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F72" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D72" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="E72" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="F72" s="6" t="s">
-        <v>231</v>
-      </c>
       <c r="G72" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H72" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="6"/>
@@ -3813,25 +3813,25 @@
         <v>67</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C73" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G73" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="D73" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>234</v>
-      </c>
       <c r="H73" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
@@ -3841,25 +3841,25 @@
         <v>68</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C74" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="G74" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="D74" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="G74" s="7" t="s">
-        <v>237</v>
-      </c>
       <c r="H74" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="6"/>
@@ -3869,25 +3869,25 @@
         <v>69</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
@@ -3897,22 +3897,22 @@
         <v>70</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H76" s="7" t="s">
         <v>20</v>
@@ -3925,25 +3925,25 @@
         <v>71</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C77" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F77" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="G77" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="E77" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F77" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>249</v>
-      </c>
       <c r="H77" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
@@ -3953,67 +3953,67 @@
         <v>72</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C78" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F78" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="D78" s="7" t="s">
+      <c r="G78" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="E78" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F78" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="G78" s="7" t="s">
-        <v>253</v>
-      </c>
       <c r="H78" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="6"/>
     </row>
     <row r="79" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="B79" s="15"/>
-      <c r="C79" s="15"/>
-      <c r="D79" s="15"/>
-      <c r="E79" s="15"/>
-      <c r="F79" s="15"/>
-      <c r="G79" s="15"/>
-      <c r="H79" s="15"/>
-      <c r="I79" s="15"/>
-      <c r="J79" s="15"/>
+      <c r="A79" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="B79" s="24"/>
+      <c r="C79" s="24"/>
+      <c r="D79" s="24"/>
+      <c r="E79" s="24"/>
+      <c r="F79" s="24"/>
+      <c r="G79" s="24"/>
+      <c r="H79" s="24"/>
+      <c r="I79" s="24"/>
+      <c r="J79" s="24"/>
     </row>
     <row r="80" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>73</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="D80" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="C80" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>257</v>
-      </c>
       <c r="E80" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>63</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
@@ -4023,25 +4023,25 @@
         <v>74</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C81" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="E81" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="D81" s="7" t="s">
+      <c r="F81" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="G81" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="E81" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="F81" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G81" s="7" t="s">
-        <v>263</v>
-      </c>
       <c r="H81" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I81" s="6"/>
       <c r="J81" s="6"/>
@@ -4051,25 +4051,25 @@
         <v>75</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C82" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E82" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="D82" s="3" t="s">
+      <c r="F82" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G82" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="E82" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="G82" s="3" t="s">
-        <v>267</v>
-      </c>
       <c r="H82" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
@@ -4079,25 +4079,25 @@
         <v>76</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C83" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="G83" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="D83" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="E83" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="F83" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="G83" s="7" t="s">
-        <v>270</v>
-      </c>
       <c r="H83" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I83" s="6"/>
       <c r="J83" s="6"/>
@@ -4107,25 +4107,25 @@
         <v>77</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C84" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="E84" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="D84" s="3" t="s">
+      <c r="F84" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="E84" s="2" t="s">
+      <c r="G84" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="F84" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="G84" s="3" t="s">
-        <v>275</v>
-      </c>
       <c r="H84" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
@@ -4135,25 +4135,25 @@
         <v>78</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C85" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="G85" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="D85" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="E85" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="F85" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="G85" s="7" t="s">
-        <v>278</v>
-      </c>
       <c r="H85" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I85" s="6"/>
       <c r="J85" s="6"/>
@@ -4163,25 +4163,25 @@
         <v>79</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C86" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F86" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="D86" s="3" t="s">
+      <c r="G86" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="E86" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F86" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="G86" s="3" t="s">
-        <v>282</v>
-      </c>
       <c r="H86" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
@@ -4191,25 +4191,25 @@
         <v>80</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C87" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="G87" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="D87" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F87" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="G87" s="7" t="s">
-        <v>285</v>
-      </c>
       <c r="H87" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I87" s="6"/>
       <c r="J87" s="6"/>
@@ -4219,25 +4219,25 @@
         <v>81</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
@@ -4247,25 +4247,25 @@
         <v>82</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C89" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="G89" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="D89" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="E89" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="F89" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="G89" s="7" t="s">
-        <v>291</v>
-      </c>
       <c r="H89" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I89" s="6"/>
       <c r="J89" s="6"/>
@@ -4275,25 +4275,25 @@
         <v>83</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C90" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F90" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="G90" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="E90" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="G90" s="3" t="s">
-        <v>295</v>
-      </c>
       <c r="H90" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
@@ -4303,25 +4303,25 @@
         <v>84</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C91" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="G91" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="D91" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="E91" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="F91" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="G91" s="7" t="s">
-        <v>298</v>
-      </c>
       <c r="H91" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I91" s="6"/>
       <c r="J91" s="6"/>
@@ -4331,25 +4331,25 @@
         <v>85</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C92" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F92" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D92" s="3" t="s">
+      <c r="G92" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="E92" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="F92" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="G92" s="3" t="s">
-        <v>302</v>
-      </c>
       <c r="H92" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
@@ -4359,25 +4359,25 @@
         <v>86</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C93" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G93" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="D93" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="E93" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F93" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="G93" s="7" t="s">
-        <v>305</v>
-      </c>
       <c r="H93" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I93" s="6"/>
       <c r="J93" s="6"/>
@@ -4387,25 +4387,25 @@
         <v>87</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C94" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G94" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="D94" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="G94" s="3" t="s">
-        <v>308</v>
-      </c>
       <c r="H94" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
@@ -4415,25 +4415,25 @@
         <v>88</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C95" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="G95" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="D95" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="E95" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F95" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G95" s="7" t="s">
-        <v>311</v>
-      </c>
       <c r="H95" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I95" s="6"/>
       <c r="J95" s="6"/>
@@ -4443,25 +4443,25 @@
         <v>89</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
@@ -4471,25 +4471,25 @@
         <v>90</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E97" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F97" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="H97" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I97" s="6"/>
       <c r="J97" s="6"/>
@@ -4499,69 +4499,69 @@
         <v>91</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H98" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I98" s="4"/>
       <c r="J98" s="4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="12" t="s">
-        <v>323</v>
-      </c>
-      <c r="B99" s="13"/>
-      <c r="C99" s="13"/>
-      <c r="D99" s="13"/>
-      <c r="E99" s="13"/>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
-      <c r="H99" s="13"/>
-      <c r="I99" s="13"/>
-      <c r="J99" s="13"/>
+      <c r="A99" s="21" t="s">
+        <v>321</v>
+      </c>
+      <c r="B99" s="22"/>
+      <c r="C99" s="22"/>
+      <c r="D99" s="22"/>
+      <c r="E99" s="22"/>
+      <c r="F99" s="22"/>
+      <c r="G99" s="22"/>
+      <c r="H99" s="22"/>
+      <c r="I99" s="22"/>
+      <c r="J99" s="22"/>
     </row>
     <row r="100" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="6">
         <v>92</v>
       </c>
       <c r="B100" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="D100" s="7" t="s">
         <v>324</v>
-      </c>
-      <c r="C100" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>326</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G100" s="7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H100" s="7" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="6"/>
@@ -4571,25 +4571,25 @@
         <v>93</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I101" s="2"/>
       <c r="J101" s="2"/>
@@ -4599,25 +4599,25 @@
         <v>94</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D102" s="7" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G102" s="7" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="H102" s="7" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="6"/>
@@ -4627,25 +4627,25 @@
         <v>95</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="I103" s="2"/>
       <c r="J103" s="2"/>
@@ -4655,25 +4655,25 @@
         <v>96</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D104" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G104" s="7" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H104" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="6"/>
@@ -4683,25 +4683,25 @@
         <v>97</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I105" s="2"/>
       <c r="J105" s="2"/>
@@ -4711,25 +4711,25 @@
         <v>98</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D106" s="7" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G106" s="7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H106" s="7" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="I106" s="6"/>
       <c r="J106" s="6"/>
@@ -4739,25 +4739,25 @@
         <v>99</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="H107" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I107" s="2"/>
       <c r="J107" s="2"/>
@@ -4767,25 +4767,25 @@
         <v>100</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D108" s="7" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>63</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G108" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H108" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I108" s="6"/>
       <c r="J108" s="6"/>
@@ -4795,22 +4795,22 @@
         <v>101</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H109" s="3" t="s">
         <v>32</v>
@@ -4823,25 +4823,25 @@
         <v>102</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D110" s="7" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G110" s="7" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="H110" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I110" s="6"/>
       <c r="J110" s="6"/>
@@ -4851,25 +4851,25 @@
         <v>103</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I111" s="2"/>
       <c r="J111" s="2"/>
@@ -4879,69 +4879,69 @@
         <v>104</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E112" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G112" s="5" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H112" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I112" s="4"/>
       <c r="J112" s="4" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A113" s="18" t="s">
-        <v>367</v>
-      </c>
-      <c r="B113" s="19"/>
-      <c r="C113" s="19"/>
-      <c r="D113" s="19"/>
-      <c r="E113" s="19"/>
-      <c r="F113" s="19"/>
-      <c r="G113" s="19"/>
-      <c r="H113" s="19"/>
-      <c r="I113" s="19"/>
-      <c r="J113" s="19"/>
+      <c r="A113" s="27" t="s">
+        <v>365</v>
+      </c>
+      <c r="B113" s="28"/>
+      <c r="C113" s="28"/>
+      <c r="D113" s="28"/>
+      <c r="E113" s="28"/>
+      <c r="F113" s="28"/>
+      <c r="G113" s="28"/>
+      <c r="H113" s="28"/>
+      <c r="I113" s="28"/>
+      <c r="J113" s="28"/>
     </row>
     <row r="114" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>105</v>
       </c>
       <c r="B114" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="D114" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="C114" s="3" t="s">
+      <c r="E114" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F114" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="D114" s="3" t="s">
+      <c r="G114" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="E114" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F114" s="2" t="s">
+      <c r="H114" s="3" t="s">
         <v>371</v>
-      </c>
-      <c r="G114" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="H114" s="3" t="s">
-        <v>373</v>
       </c>
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
@@ -4951,25 +4951,25 @@
         <v>106</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C115" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F115" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="D115" s="7" t="s">
+      <c r="G115" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="E115" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F115" s="6" t="s">
-        <v>376</v>
-      </c>
-      <c r="G115" s="7" t="s">
-        <v>377</v>
-      </c>
       <c r="H115" s="7" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I115" s="6"/>
       <c r="J115" s="6"/>
@@ -4979,25 +4979,25 @@
         <v>107</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I116" s="2"/>
       <c r="J116" s="2"/>
@@ -5007,25 +5007,25 @@
         <v>108</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G117" s="7" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="H117" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I117" s="6"/>
       <c r="J117" s="6"/>
@@ -5035,22 +5035,22 @@
         <v>109</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="H118" s="3" t="s">
         <v>25</v>
@@ -5063,22 +5063,22 @@
         <v>110</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D119" s="7" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>44</v>
       </c>
       <c r="F119" s="6" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="G119" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="H119" s="7" t="s">
         <v>20</v>
@@ -5088,6 +5088,7 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A113:J113"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A63:J63"/>
@@ -5095,7 +5096,6 @@
     <mergeCell ref="A99:J99"/>
     <mergeCell ref="A79:J79"/>
     <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A113:J113"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5113,119 +5113,119 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>393</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B2" s="2">
         <v>36</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B3" s="2">
         <v>118</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B4" s="2">
         <v>126</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>406</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B6" s="2">
         <v>36</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="8" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -5253,13 +5253,13 @@
         <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>414</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -5267,16 +5267,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>418</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -5284,16 +5284,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>422</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="25" x14ac:dyDescent="0.35">
@@ -5301,16 +5301,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>425</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>426</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" x14ac:dyDescent="0.35">
@@ -5318,16 +5318,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>429</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -5335,16 +5335,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -5352,16 +5352,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>434</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Homepage redesign, ScrollReveal primitive, visual polish across components
- Redesign homepage with scroll-reveal animations and updated section layout
- Add ScrollReveal primitive for intersection-observer-based entrance animations
- Enhance HomepageHero, HowItWorks, TrustSignals, TestimonialCarousel components
- Update CTABlock, ComplianceCallout, PillarCard with improved styling
- Add CSS animations (fade-in, slide-up, scale-in) to globals.css
- Update .gitignore to exclude audit screenshots and playwright-mcp

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOCS/Incorporate123_Project_Task_List.xlsx
+++ b/DOCS/Incorporate123_Project_Task_List.xlsx
@@ -1500,6 +1500,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1528,10 +1532,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1881,18 +1881,18 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
     </row>
     <row r="3" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10">
@@ -2205,18 +2205,18 @@
       <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
     </row>
     <row r="15" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
@@ -2585,18 +2585,18 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
     </row>
     <row r="29" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="10">
@@ -3019,18 +3019,18 @@
       <c r="J43" s="2"/>
     </row>
     <row r="44" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
+      <c r="B44" s="22"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
+      <c r="I44" s="22"/>
+      <c r="J44" s="22"/>
     </row>
     <row r="45" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6">
@@ -3543,18 +3543,18 @@
       </c>
     </row>
     <row r="63" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="17" t="s">
+      <c r="A63" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="B63" s="18"/>
-      <c r="C63" s="18"/>
-      <c r="D63" s="18"/>
-      <c r="E63" s="18"/>
-      <c r="F63" s="18"/>
-      <c r="G63" s="18"/>
-      <c r="H63" s="18"/>
-      <c r="I63" s="18"/>
-      <c r="J63" s="18"/>
+      <c r="B63" s="20"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="20"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="20"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
     </row>
     <row r="64" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6">
@@ -3977,18 +3977,18 @@
       <c r="J78" s="6"/>
     </row>
     <row r="79" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="23" t="s">
+      <c r="A79" s="25" t="s">
         <v>252</v>
       </c>
-      <c r="B79" s="24"/>
-      <c r="C79" s="24"/>
-      <c r="D79" s="24"/>
-      <c r="E79" s="24"/>
-      <c r="F79" s="24"/>
-      <c r="G79" s="24"/>
-      <c r="H79" s="24"/>
-      <c r="I79" s="24"/>
-      <c r="J79" s="24"/>
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
+      <c r="F79" s="26"/>
+      <c r="G79" s="26"/>
+      <c r="H79" s="26"/>
+      <c r="I79" s="26"/>
+      <c r="J79" s="26"/>
     </row>
     <row r="80" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
@@ -4525,18 +4525,18 @@
       </c>
     </row>
     <row r="99" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="21" t="s">
+      <c r="A99" s="23" t="s">
         <v>321</v>
       </c>
-      <c r="B99" s="22"/>
-      <c r="C99" s="22"/>
-      <c r="D99" s="22"/>
-      <c r="E99" s="22"/>
-      <c r="F99" s="22"/>
-      <c r="G99" s="22"/>
-      <c r="H99" s="22"/>
-      <c r="I99" s="22"/>
-      <c r="J99" s="22"/>
+      <c r="B99" s="24"/>
+      <c r="C99" s="24"/>
+      <c r="D99" s="24"/>
+      <c r="E99" s="24"/>
+      <c r="F99" s="24"/>
+      <c r="G99" s="24"/>
+      <c r="H99" s="24"/>
+      <c r="I99" s="24"/>
+      <c r="J99" s="24"/>
     </row>
     <row r="100" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="6">
@@ -4905,18 +4905,18 @@
       </c>
     </row>
     <row r="113" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A113" s="27" t="s">
+      <c r="A113" s="13" t="s">
         <v>365</v>
       </c>
-      <c r="B113" s="28"/>
-      <c r="C113" s="28"/>
-      <c r="D113" s="28"/>
-      <c r="E113" s="28"/>
-      <c r="F113" s="28"/>
-      <c r="G113" s="28"/>
-      <c r="H113" s="28"/>
-      <c r="I113" s="28"/>
-      <c r="J113" s="28"/>
+      <c r="B113" s="14"/>
+      <c r="C113" s="14"/>
+      <c r="D113" s="14"/>
+      <c r="E113" s="14"/>
+      <c r="F113" s="14"/>
+      <c r="G113" s="14"/>
+      <c r="H113" s="14"/>
+      <c r="I113" s="14"/>
+      <c r="J113" s="14"/>
     </row>
     <row r="114" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="2">

</xml_diff>

<commit_message>
Reorganize DOCS: move meeting preps, deliverables, add page specs and blueprint
- Move meeting prep files to DOCS/Meeting Preps/
- Move Phase 1 final deliverables to subfolder 8
- Move finalization docs to subfolder 9
- Add 20 page specifications for all page types (00-19)
- Add pillar page v10 blueprint for replicating redesign
- Add enhanced pillar page specifications (Privacy, Asset, Formation, Compliance)
- Remove old prototype/ directory (replaced by inc123-prototype/)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOCS/Incorporate123_Project_Task_List.xlsx
+++ b/DOCS/Incorporate123_Project_Task_List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexo\Projects\inc123\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE8FC8E-4228-4FFE-81D8-8BF19405EBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CC82E8-7FF1-4BB5-AC96-3B6F32DE4AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1464,7 +1464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1532,6 +1532,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2526,61 +2532,61 @@
       <c r="I25" s="10"/>
       <c r="J25" s="10"/>
     </row>
-    <row r="26" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="2">
+    <row r="26" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="10">
         <v>23</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="H26" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-    </row>
-    <row r="27" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="4">
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+    </row>
+    <row r="27" spans="1:10" s="12" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="29">
         <v>24</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="G27" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="5" t="s">
+      <c r="H27" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4" t="s">
+      <c r="I27" s="29"/>
+      <c r="J27" s="29" t="s">
         <v>94</v>
       </c>
     </row>

</xml_diff>